<commit_message>
check wrong format import and export excel completion rate service
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportCompleteRate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportCompleteRate.xlsx
@@ -32,8 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -108,12 +109,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -134,52 +139,20 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="12.640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.5"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-    </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-    </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>